<commit_message>
Rewritten PCD - initial setup utils
- Updated hydrophone sheets - wrong unit
- acquire_data not private anymore
- remove bugs
</commit_message>
<xml_diff>
--- a/SonoRover One/software/src/config/hydrophones/HGL 0200 SN2845 Calibration datasheet.xlsx
+++ b/SonoRover One/software/src/config/hydrophones/HGL 0200 SN2845 Calibration datasheet.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitLab\Radboud-FUS-measurement-kit\SonoRover One\software\src\config\hydrophones\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/Software/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/src/config/hydrophones/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_2222E724495BD25E9F6948D5F3E9B3AA0762BBDA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{842C71C0-DDBB-4BC2-A09C-709A68E9719E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -18,6 +19,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -35,11 +47,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.000000000"/>
+    <numFmt numFmtId="168" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +102,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -408,14 +424,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="32.5" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -423,147 +439,147 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0.25</v>
       </c>
       <c r="B2" s="3">
-        <v>2.2949999999999999E-4</v>
+        <v>2.2950000000000001E-7</v>
       </c>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>0.3</v>
       </c>
       <c r="B3" s="3">
-        <v>2.7169999999999999E-4</v>
+        <v>2.7169999999999998E-7</v>
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>0.35</v>
       </c>
       <c r="B4" s="3">
-        <v>2.6269999999999999E-4</v>
+        <v>2.6269999999999999E-7</v>
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>0.4</v>
       </c>
       <c r="B5" s="3">
-        <v>2.6830000000000002E-4</v>
+        <v>2.6829999999999999E-7</v>
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>0.45</v>
       </c>
       <c r="B6" s="3">
-        <v>2.6570000000000001E-4</v>
+        <v>2.657E-7</v>
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>0.5</v>
       </c>
       <c r="B7" s="3">
-        <v>2.542E-4</v>
+        <v>2.5419999999999999E-7</v>
       </c>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>0.55000000000000004</v>
       </c>
       <c r="B8" s="3">
-        <v>2.5099999999999998E-4</v>
+        <v>2.5100000000000001E-7</v>
       </c>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>0.6</v>
       </c>
       <c r="B9" s="3">
-        <v>2.4669999999999998E-4</v>
+        <v>2.4670000000000001E-7</v>
       </c>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>0.65</v>
       </c>
       <c r="B10" s="3">
-        <v>2.4360000000000001E-4</v>
+        <v>2.4359999999999998E-7</v>
       </c>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>0.7</v>
       </c>
       <c r="B11" s="3">
-        <v>2.365E-4</v>
+        <v>2.3650000000000001E-7</v>
       </c>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>0.75</v>
       </c>
       <c r="B12" s="3">
-        <v>2.2680000000000001E-4</v>
+        <v>2.2679999999999999E-7</v>
       </c>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>0.8</v>
       </c>
       <c r="B13" s="3">
-        <v>2.218E-4</v>
+        <v>2.2179999999999999E-7</v>
       </c>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>0.85</v>
       </c>
       <c r="B14" s="3">
-        <v>2.141E-4</v>
+        <v>2.1409999999999999E-7</v>
       </c>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>0.9</v>
       </c>
       <c r="B15" s="3">
-        <v>2.052E-4</v>
+        <v>2.0520000000000001E-7</v>
       </c>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>0.95</v>
       </c>
       <c r="B16" s="3">
-        <v>1.9770000000000001E-4</v>
+        <v>1.977E-7</v>
       </c>
       <c r="D16" s="1"/>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>1</v>
       </c>
       <c r="B17" s="3">
-        <v>1.8929999999999999E-4</v>
+        <v>1.8930000000000001E-7</v>
       </c>
       <c r="D17" s="1"/>
     </row>

</xml_diff>